<commit_message>
ENOS: automatizar cortes y cambios parciales, conservando la última carga validada ante errores
</commit_message>
<xml_diff>
--- a/data/enos_excel/unidades_suspendidas.xlsx
+++ b/data/enos_excel/unidades_suspendidas.xlsx
@@ -2,10 +2,32 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="1" r:id="Radadf44d8f30486b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R2543b5e1ea964c91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="1" r:id="Rd33c9655845242cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R97d14b9948f04ebf"/>
   </x:sheets>
 </x:workbook>
+</file>
+
+<file path=xl/metadata1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:metadata xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:metadataTypes count="1">
+    <x:metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </x:metadataTypes>
+  <x:futureMetadata name="XLDAPR" count="1">
+    <x:bk>
+      <x:extLst>
+        <x:ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" fDynamic="1" fCollapsed="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:bk>
+  </x:futureMetadata>
+  <x:cellMetadata count="1">
+    <x:bk>
+      <x:rc t="1" v="0"/>
+    </x:bk>
+  </x:cellMetadata>
+</x:metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -74,9 +96,6 @@
     <x:t xml:space="preserve">corte</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Actualizar al corte de la fuente antes de cargar datos de fechas posteriores.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">publicacion_base</x:t>
   </x:si>
   <x:si>
@@ -110,31 +129,16 @@
     <x:t xml:space="preserve">Paso 1</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Cada corte debe contener el inventario completo de unidades con suspensión.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Paso 2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Para un corte nuevo, copia todas las filas del corte vigente y cambia corte_fuente.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Paso 3</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Conserva id_unidad. Marca Reanudada cuando una unidad vuelva a atender; agrega las nuevas unidades.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Paso 4</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Actualiza corte en B4. El sistema usa un solo corte, nunca la suma de cortes.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Último corte</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Suspendidas del corte</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Campo</x:t>
@@ -229,7 +233,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -251,6 +255,11 @@
         <x:fgColor rgb="FFEAE3F3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAE3F3"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -264,7 +273,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -291,6 +300,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="165" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -19886,7 +19898,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd68e96eedfaa471d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc37d0d813fc64a6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19940,44 +19952,45 @@
       <x:c r="A4" s="1" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B4" s="13">
+      <x:c r="B4" s="14" t="n">
+        <x:f>MAX(Datos!B:B)</x:f>
         <x:v>46324</x:v>
       </x:c>
-      <x:c r="C4" s="11" t="s">
-        <x:v>21</x:v>
+      <x:c r="C4" s="11" t="str">
+        <x:v>Automático a partir de las fechas de Datos. No editar.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B5" s="11" t="s">
+      <x:c r="C5" s="11" t="s">
         <x:v>23</x:v>
-      </x:c>
-      <x:c r="C5" s="11" t="s">
-        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="1" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B6" s="11" t="s">
+      <x:c r="C6" s="11" t="s">
         <x:v>26</x:v>
-      </x:c>
-      <x:c r="C6" s="11" t="s">
-        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="1" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B7" s="11" t="s">
+      <x:c r="C7" s="11" t="s">
         <x:v>29</x:v>
-      </x:c>
-      <x:c r="C7" s="11" t="s">
-        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -19987,45 +20000,45 @@
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="7" t="s">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B9" s="1"/>
       <x:c r="C9" s="11"/>
     </x:row>
     <x:row r="10" ht="40" customHeight="1">
       <x:c r="A10" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B10" s="1"/>
-      <x:c r="C10" s="11" t="s">
-        <x:v>33</x:v>
+      <x:c r="C10" s="11" t="str">
+        <x:v>Para un reporte nuevo, agrega solo las filas de las unidades que cambiaron.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40" customHeight="1">
       <x:c r="A11" s="1" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B11" s="1"/>
-      <x:c r="C11" s="11" t="s">
-        <x:v>35</x:v>
+      <x:c r="C11" s="11" t="str">
+        <x:v>Conserva id_unidad y escribe la fecha real del reporte en corte_fuente.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" customHeight="1">
       <x:c r="A12" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B12" s="1"/>
-      <x:c r="C12" s="11" t="s">
-        <x:v>37</x:v>
+      <x:c r="C12" s="11" t="str">
+        <x:v>Marca Reanudada al volver a atender. Las demás unidades conservan su último estado.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="40" customHeight="1">
       <x:c r="A13" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B13" s="1"/>
-      <x:c r="C13" s="11" t="s">
-        <x:v>39</x:v>
+      <x:c r="C13" s="11" t="str">
+        <x:v>No copies todo el inventario. Guarda y sube el archivo; el tablero reconstruye el stock automáticamente.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -20035,7 +20048,7 @@
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
       <x:c r="A15" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B15" s="8" t="n">
         <x:f>MAX(Datos!B:B)</x:f>
@@ -20044,11 +20057,11 @@
       <x:c r="C15" s="11"/>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
-      <x:c r="A16" s="1" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B16" s="9" t="n">
-        <x:f>COUNTIFS(Datos!B:B,B15,Datos!K:K,"&lt;&gt;Reanudada")</x:f>
+      <x:c r="A16" s="1" t="str">
+        <x:v>Suspendidas vigentes</x:v>
+      </x:c>
+      <x:c r="B16" s="9" t="n" cm="1">
+        <x:f t="array" ref="B16">SUM(_xlfn.BYROW(_xlfn.UNIQUE(Unidades[id_unidad]),_xlfn.LAMBDA(_xlpm.id,COUNTIFS(Unidades[id_unidad],_xlpm.id,Unidades[corte_fuente],_xlfn.MAXIFS(Unidades[corte_fuente],Unidades[id_unidad],_xlpm.id),Unidades[estado],"&lt;&gt;Reanudada"))))</x:f>
         <x:v>119</x:v>
       </x:c>
       <x:c r="C16" s="11"/>
@@ -20070,13 +20083,13 @@
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
       <x:c r="A20" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B20" s="10" t="s">
-        <x:v>43</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="C20" s="12" t="s">
-        <x:v>44</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
@@ -20084,10 +20097,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B21" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C21" s="11" t="s">
-        <x:v>46</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
@@ -20095,10 +20108,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B22" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C22" s="11" t="s">
-        <x:v>48</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
@@ -20106,10 +20119,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B23" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C23" s="11" t="s">
-        <x:v>49</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
@@ -20117,10 +20130,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C24" s="11" t="s">
-        <x:v>50</x:v>
+        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="34" customHeight="1">
@@ -20128,10 +20141,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B25" s="1" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="C25" s="11" t="s">
         <x:v>45</x:v>
-      </x:c>
-      <x:c r="C25" s="11" t="s">
-        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="34" customHeight="1">
@@ -20139,10 +20152,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B26" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C26" s="11" t="s">
-        <x:v>52</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="34" customHeight="1">
@@ -20150,10 +20163,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B27" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C27" s="11" t="s">
-        <x:v>53</x:v>
+        <x:v>47</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="34" customHeight="1">
@@ -20161,10 +20174,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B28" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C28" s="11" t="s">
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="34" customHeight="1">
@@ -20172,10 +20185,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B29" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C29" s="11" t="s">
-        <x:v>55</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="34" customHeight="1">
@@ -20183,10 +20196,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B30" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C30" s="11" t="s">
-        <x:v>56</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="34" customHeight="1">
@@ -20194,10 +20207,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B31" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C31" s="11" t="s">
-        <x:v>57</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
@@ -20205,10 +20218,10 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B32" s="1" t="s">
-        <x:v>58</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C32" s="11" t="s">
-        <x:v>59</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="34" customHeight="1">

</xml_diff>